<commit_message>
final code for Italy and Working fine.
</commit_message>
<xml_diff>
--- a/Data/Hungary_New Hire_Store 970_automationFileM - Copy (5).xlsx
+++ b/Data/Hungary_New Hire_Store 970_automationFileM - Copy (5).xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E4FA84E-A547-457E-A69F-DF4C443A6D54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14827326-2B6C-45FC-A9B9-5EF640088980}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4140,7 +4140,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4227,6 +4227,20 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -4286,7 +4300,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -4457,6 +4471,45 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="15" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4737,7 +4790,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:CU77"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="14.5" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
@@ -5113,7 +5165,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="35" t="s">
         <v>94</v>
       </c>
@@ -5418,7 +5470,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="3" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="35" t="s">
         <v>151</v>
       </c>
@@ -5724,7 +5776,7 @@
         <v>123456015</v>
       </c>
     </row>
-    <row r="4" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="35" t="s">
         <v>162</v>
       </c>
@@ -6029,7 +6081,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="5" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="35" t="s">
         <v>166</v>
       </c>
@@ -6335,7 +6387,7 @@
         <v>123456016</v>
       </c>
     </row>
-    <row r="6" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="35" t="s">
         <v>171</v>
       </c>
@@ -7251,7 +7303,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="9" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="35" t="s">
         <v>185</v>
       </c>
@@ -8778,7 +8830,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="14" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="35" t="s">
         <v>206</v>
       </c>
@@ -9083,7 +9135,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="15" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="35" t="s">
         <v>213</v>
       </c>
@@ -10000,7 +10052,7 @@
         <v>123456020</v>
       </c>
     </row>
-    <row r="18" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="35" t="s">
         <v>224</v>
       </c>
@@ -10610,7 +10662,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="20" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="35" t="s">
         <v>232</v>
       </c>
@@ -10915,7 +10967,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="21" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="35" t="s">
         <v>240</v>
       </c>
@@ -11527,7 +11579,7 @@
         <v>123456085</v>
       </c>
     </row>
-    <row r="23" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="35" t="s">
         <v>247</v>
       </c>
@@ -11833,7 +11885,7 @@
         <v>123456022</v>
       </c>
     </row>
-    <row r="24" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="35" t="s">
         <v>251</v>
       </c>
@@ -13666,7 +13718,7 @@
         <v>123456024</v>
       </c>
     </row>
-    <row r="30" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="35" t="s">
         <v>278</v>
       </c>
@@ -13971,111 +14023,111 @@
         <v>113</v>
       </c>
     </row>
-    <row r="31" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="35" t="s">
+    <row r="31" spans="1:99" s="72" customFormat="1" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="61" t="s">
         <v>282</v>
       </c>
-      <c r="B31" s="35" t="s">
+      <c r="B31" s="61" t="s">
         <v>283</v>
       </c>
-      <c r="C31" s="35" t="s">
+      <c r="C31" s="61" t="s">
         <v>177</v>
       </c>
       <c r="D31" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="E31" s="38" t="s">
-        <v>97</v>
-      </c>
-      <c r="F31" s="39" t="s">
+      <c r="E31" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="F31" s="62" t="s">
         <v>284</v>
       </c>
-      <c r="G31" s="39" t="s">
+      <c r="G31" s="62" t="s">
         <v>491</v>
       </c>
-      <c r="H31" s="40" t="s">
+      <c r="H31" s="63" t="s">
         <v>100</v>
       </c>
-      <c r="I31" s="40" t="s">
+      <c r="I31" s="63" t="s">
         <v>101</v>
       </c>
-      <c r="J31" s="40" t="s">
+      <c r="J31" s="63" t="s">
         <v>102</v>
       </c>
       <c r="K31" s="41">
         <f t="shared" si="3"/>
         <v>45658</v>
       </c>
-      <c r="L31" s="38" t="s">
-        <v>97</v>
-      </c>
-      <c r="M31" s="40" t="s">
+      <c r="L31" s="37" t="s">
+        <v>97</v>
+      </c>
+      <c r="M31" s="63" t="s">
         <v>103</v>
       </c>
-      <c r="N31" s="40" t="s">
+      <c r="N31" s="63" t="s">
         <v>153</v>
       </c>
-      <c r="O31" s="42" t="s">
+      <c r="O31" s="63" t="s">
         <v>105</v>
       </c>
-      <c r="P31" s="38" t="s">
+      <c r="P31" s="37" t="s">
         <v>154</v>
       </c>
-      <c r="Q31" s="40" t="s">
+      <c r="Q31" s="63" t="s">
         <v>107</v>
       </c>
-      <c r="R31" s="40" t="s">
+      <c r="R31" s="63" t="s">
         <v>108</v>
       </c>
-      <c r="S31" s="43" t="s">
+      <c r="S31" s="64" t="s">
         <v>109</v>
       </c>
-      <c r="T31" s="43" t="s">
+      <c r="T31" s="64" t="s">
         <v>109</v>
       </c>
-      <c r="U31" s="40" t="s">
+      <c r="U31" s="63" t="s">
         <v>102</v>
       </c>
-      <c r="V31" s="44" t="s">
+      <c r="V31" s="41" t="s">
         <v>110</v>
       </c>
-      <c r="W31" s="45" t="s">
+      <c r="W31" s="65" t="s">
         <v>111</v>
       </c>
-      <c r="X31" s="40" t="s">
+      <c r="X31" s="63" t="s">
         <v>102</v>
       </c>
       <c r="Y31" s="46">
         <v>45658</v>
       </c>
-      <c r="Z31" s="40" t="s">
+      <c r="Z31" s="63" t="s">
         <v>112</v>
       </c>
-      <c r="AA31" s="47" t="s">
-        <v>113</v>
-      </c>
-      <c r="AB31" s="48" t="s">
+      <c r="AA31" s="66" t="s">
+        <v>113</v>
+      </c>
+      <c r="AB31" s="62" t="s">
         <v>236</v>
       </c>
-      <c r="AC31" s="48" t="s">
+      <c r="AC31" s="62" t="s">
         <v>263</v>
       </c>
-      <c r="AD31" s="39" t="s">
+      <c r="AD31" s="62" t="s">
         <v>116</v>
       </c>
-      <c r="AE31" s="38">
+      <c r="AE31" s="37">
         <v>970</v>
       </c>
-      <c r="AF31" s="38" t="s">
+      <c r="AF31" s="37" t="s">
         <v>57</v>
       </c>
-      <c r="AG31" s="39">
+      <c r="AG31" s="62">
         <v>25</v>
       </c>
-      <c r="AH31" s="49" t="s">
+      <c r="AH31" s="62" t="s">
         <v>169</v>
       </c>
-      <c r="AI31" s="48" t="s">
+      <c r="AI31" s="62" t="s">
         <v>118</v>
       </c>
       <c r="AJ31" s="46" t="s">
@@ -14085,45 +14137,45 @@
         <f t="shared" si="0"/>
         <v>45748</v>
       </c>
-      <c r="AL31" s="40" t="s">
+      <c r="AL31" s="63" t="s">
         <v>119</v>
       </c>
-      <c r="AM31" s="49" t="s">
+      <c r="AM31" s="62" t="s">
         <v>120</v>
       </c>
-      <c r="AN31" s="39" t="s">
+      <c r="AN31" s="62" t="s">
         <v>264</v>
       </c>
-      <c r="AO31" s="40" t="s">
+      <c r="AO31" s="63" t="s">
         <v>122</v>
       </c>
-      <c r="AP31" s="50" t="s">
+      <c r="AP31" s="37" t="s">
         <v>123</v>
       </c>
-      <c r="AQ31" s="40" t="s">
+      <c r="AQ31" s="63" t="s">
         <v>124</v>
       </c>
-      <c r="AR31" s="35" t="s">
+      <c r="AR31" s="61" t="s">
         <v>124</v>
       </c>
-      <c r="AS31" s="44" t="s">
-        <v>113</v>
-      </c>
-      <c r="AT31" s="40" t="s">
+      <c r="AS31" s="41" t="s">
+        <v>113</v>
+      </c>
+      <c r="AT31" s="63" t="s">
         <v>125</v>
       </c>
-      <c r="AU31" s="50" t="str">
+      <c r="AU31" s="37" t="str">
         <f t="shared" si="6"/>
         <v>Permanent</v>
       </c>
-      <c r="AV31" s="44" t="s">
+      <c r="AV31" s="41" t="s">
         <v>127</v>
       </c>
-      <c r="AW31" s="51">
+      <c r="AW31" s="41">
         <f t="shared" si="5"/>
         <v>45657</v>
       </c>
-      <c r="AX31" s="51">
+      <c r="AX31" s="41">
         <f t="shared" si="1"/>
         <v>45657</v>
       </c>
@@ -14131,152 +14183,152 @@
         <f t="shared" si="2"/>
         <v>N/A</v>
       </c>
-      <c r="AZ31" s="43" t="s">
-        <v>97</v>
-      </c>
-      <c r="BA31" s="43" t="s">
+      <c r="AZ31" s="64" t="s">
+        <v>97</v>
+      </c>
+      <c r="BA31" s="64" t="s">
         <v>128</v>
       </c>
-      <c r="BB31" s="52" t="s">
+      <c r="BB31" s="67" t="s">
         <v>285</v>
       </c>
-      <c r="BC31" s="44">
+      <c r="BC31" s="41">
         <v>36526</v>
       </c>
-      <c r="BD31" s="44">
+      <c r="BD31" s="41">
         <v>51136</v>
       </c>
-      <c r="BE31" s="43" t="s">
-        <v>97</v>
-      </c>
-      <c r="BF31" s="43" t="s">
+      <c r="BE31" s="64" t="s">
+        <v>97</v>
+      </c>
+      <c r="BF31" s="64" t="s">
         <v>132</v>
       </c>
-      <c r="BG31" s="50">
+      <c r="BG31" s="37">
         <v>5855200059</v>
       </c>
-      <c r="BH31" s="44">
+      <c r="BH31" s="41">
         <v>36526</v>
       </c>
-      <c r="BI31" s="44">
+      <c r="BI31" s="41">
         <v>51136</v>
       </c>
-      <c r="BJ31" s="38" t="s">
+      <c r="BJ31" s="37" t="s">
         <v>133</v>
       </c>
-      <c r="BK31" s="50" t="s">
+      <c r="BK31" s="37" t="s">
         <v>156</v>
       </c>
-      <c r="BL31" s="53">
+      <c r="BL31" s="46">
         <v>28857</v>
       </c>
-      <c r="BM31" s="54" t="s">
-        <v>97</v>
-      </c>
-      <c r="BN31" s="43" t="s">
+      <c r="BM31" s="68" t="s">
+        <v>97</v>
+      </c>
+      <c r="BN31" s="64" t="s">
         <v>109</v>
       </c>
-      <c r="BO31" s="38" t="s">
+      <c r="BO31" s="37" t="s">
         <v>135</v>
       </c>
-      <c r="BP31" s="55" t="s">
-        <v>113</v>
-      </c>
-      <c r="BQ31" s="43" t="s">
+      <c r="BP31" s="69" t="s">
+        <v>113</v>
+      </c>
+      <c r="BQ31" s="64" t="s">
         <v>136</v>
       </c>
-      <c r="BR31" s="43" t="s">
-        <v>97</v>
-      </c>
-      <c r="BS31" s="39" t="s">
+      <c r="BR31" s="64" t="s">
+        <v>97</v>
+      </c>
+      <c r="BS31" s="62" t="s">
         <v>123</v>
       </c>
-      <c r="BT31" s="39">
+      <c r="BT31" s="62">
         <v>20</v>
       </c>
-      <c r="BU31" s="38" t="s">
+      <c r="BU31" s="37" t="s">
         <v>137</v>
       </c>
-      <c r="BV31" s="38" t="s">
+      <c r="BV31" s="37" t="s">
         <v>138</v>
       </c>
-      <c r="BW31" s="43" t="s">
+      <c r="BW31" s="64" t="s">
         <v>139</v>
       </c>
-      <c r="BX31" s="56" t="s">
+      <c r="BX31" s="70" t="s">
         <v>157</v>
       </c>
-      <c r="BY31" s="43" t="s">
+      <c r="BY31" s="64" t="s">
         <v>141</v>
       </c>
-      <c r="BZ31" s="43" t="s">
+      <c r="BZ31" s="64" t="s">
         <v>142</v>
       </c>
-      <c r="CA31" s="43" t="s">
+      <c r="CA31" s="64" t="s">
         <v>143</v>
       </c>
-      <c r="CB31" s="43" t="s">
+      <c r="CB31" s="64" t="s">
         <v>144</v>
       </c>
-      <c r="CC31" s="56" t="s">
+      <c r="CC31" s="70" t="s">
         <v>139</v>
       </c>
-      <c r="CD31" s="40" t="s">
+      <c r="CD31" s="63" t="s">
         <v>140</v>
       </c>
-      <c r="CE31" s="43" t="s">
+      <c r="CE31" s="64" t="s">
         <v>141</v>
       </c>
-      <c r="CF31" s="43" t="s">
+      <c r="CF31" s="64" t="s">
         <v>145</v>
       </c>
-      <c r="CG31" s="43" t="s">
+      <c r="CG31" s="64" t="s">
         <v>146</v>
       </c>
-      <c r="CH31" s="43" t="s">
+      <c r="CH31" s="64" t="s">
         <v>145</v>
       </c>
-      <c r="CI31" s="57">
+      <c r="CI31" s="71">
         <v>100</v>
       </c>
-      <c r="CJ31" s="43" t="s">
+      <c r="CJ31" s="64" t="s">
         <v>147</v>
       </c>
-      <c r="CK31" s="43" t="s">
+      <c r="CK31" s="64" t="s">
         <v>148</v>
       </c>
-      <c r="CL31" s="43" t="s">
-        <v>97</v>
-      </c>
-      <c r="CM31" s="43" t="s">
+      <c r="CL31" s="64" t="s">
+        <v>97</v>
+      </c>
+      <c r="CM31" s="64" t="s">
         <v>158</v>
       </c>
-      <c r="CN31" s="43" t="s">
+      <c r="CN31" s="64" t="s">
         <v>150</v>
       </c>
-      <c r="CO31" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="CP31" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="CQ31" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="CR31" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="CS31" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="CT31" s="39" t="s">
-        <v>113</v>
-      </c>
-      <c r="CU31" s="39" t="s">
+      <c r="CO31" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="CP31" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="CQ31" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="CR31" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="CS31" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="CT31" s="62" t="s">
+        <v>113</v>
+      </c>
+      <c r="CU31" s="62" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="32" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A32" s="35" t="s">
         <v>286</v>
       </c>
@@ -14581,7 +14633,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="33" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="35" t="s">
         <v>297</v>
       </c>
@@ -14887,7 +14939,7 @@
         <v>123456025</v>
       </c>
     </row>
-    <row r="34" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A34" s="35" t="s">
         <v>302</v>
       </c>
@@ -15192,7 +15244,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="35" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A35" s="35" t="s">
         <v>309</v>
       </c>
@@ -15803,7 +15855,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="37" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="35" t="s">
         <v>321</v>
       </c>
@@ -16720,7 +16772,7 @@
         <v>123456027</v>
       </c>
     </row>
-    <row r="40" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="35" t="s">
         <v>337</v>
       </c>
@@ -17331,7 +17383,7 @@
         <v>123456028</v>
       </c>
     </row>
-    <row r="42" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A42" s="35" t="s">
         <v>349</v>
       </c>
@@ -17636,7 +17688,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="43" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A43" s="35" t="s">
         <v>356</v>
       </c>
@@ -17942,7 +17994,7 @@
         <v>123456048</v>
       </c>
     </row>
-    <row r="44" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A44" s="35" t="s">
         <v>361</v>
       </c>
@@ -18247,7 +18299,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="45" spans="1:99" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:99" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="35" t="s">
         <v>368</v>
       </c>
@@ -28282,13 +28334,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:CU77" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="Failed"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:CU77" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="68">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AV10 Z10 X10 U10 I10:J10 CC10 BW10" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>INDIRECT($C2)</formula1>
@@ -28574,6 +28620,6 @@
     <hyperlink ref="W57" r:id="rId76" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId77"/>
 </worksheet>
 </file>
</xml_diff>